<commit_message>
removed electrical demand uncertainty in the run files, and in the models.py
</commit_message>
<xml_diff>
--- a/outputs/EH1_stc_results_2026-05-20.xlsx
+++ b/outputs/EH1_stc_results_2026-05-20.xlsx
@@ -690,7 +690,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>68.551</v>
+        <v>68.483</v>
       </c>
       <c r="E5" t="n">
         <v>38.078</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>15.45</v>
+        <v>15.38061224489796</v>
       </c>
       <c r="L5" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M5" t="n">
         <v>42.30888888888889</v>
@@ -849,7 +849,7 @@
         <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>75.066</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E8" t="n">
         <v>48.821</v>
@@ -861,19 +861,19 @@
         <v>79</v>
       </c>
       <c r="H8" t="n">
-        <v>76.59795918367347</v>
+        <v>79</v>
       </c>
       <c r="I8" t="n">
-        <v>2.402040816326533</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>6.834693877551018</v>
       </c>
       <c r="L8" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M8" t="n">
         <v>54.24555555555555</v>
@@ -1008,7 +1008,7 @@
         <v>10</v>
       </c>
       <c r="D11" t="n">
-        <v>125.853</v>
+        <v>138.408</v>
       </c>
       <c r="E11" t="n">
         <v>45.383</v>
@@ -1026,13 +1026,13 @@
         <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>128.4214285714286</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M11" t="n">
         <v>50.42555555555556</v>
@@ -1073,13 +1073,13 @@
         <v>34</v>
       </c>
       <c r="H12" t="n">
-        <v>21.91836734693877</v>
+        <v>0.5</v>
       </c>
       <c r="I12" t="n">
-        <v>12.08163265306123</v>
+        <v>33.5</v>
       </c>
       <c r="J12" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -1126,13 +1126,13 @@
         <v>34</v>
       </c>
       <c r="H13" t="n">
-        <v>24.43877551020408</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>9.561224489795919</v>
+        <v>33</v>
       </c>
       <c r="J13" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1167,7 +1167,7 @@
         <v>13</v>
       </c>
       <c r="D14" t="n">
-        <v>139.087</v>
+        <v>136.236</v>
       </c>
       <c r="E14" t="n">
         <v>56.911</v>
@@ -1179,19 +1179,19 @@
         <v>35</v>
       </c>
       <c r="H14" t="n">
-        <v>27.19081632653061</v>
+        <v>1.5</v>
       </c>
       <c r="I14" t="n">
-        <v>7.809183673469391</v>
+        <v>33.5</v>
       </c>
       <c r="J14" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>141.9255102040816</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M14" t="n">
         <v>63.23444444444445</v>
@@ -1232,13 +1232,13 @@
         <v>54.5</v>
       </c>
       <c r="H15" t="n">
-        <v>24.28163265306122</v>
+        <v>3.5</v>
       </c>
       <c r="I15" t="n">
-        <v>30.21836734693878</v>
+        <v>51</v>
       </c>
       <c r="J15" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1326,7 +1326,7 @@
         <v>16</v>
       </c>
       <c r="D17" t="n">
-        <v>122.799</v>
+        <v>140.444</v>
       </c>
       <c r="E17" t="n">
         <v>41.57</v>
@@ -1338,19 +1338,19 @@
         <v>163</v>
       </c>
       <c r="H17" t="n">
-        <v>4.761224489795921</v>
+        <v>11</v>
       </c>
       <c r="I17" t="n">
-        <v>158.2387755102041</v>
+        <v>152</v>
       </c>
       <c r="J17" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>125.3051020408163</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M17" t="n">
         <v>46.18888888888889</v>
@@ -1391,13 +1391,13 @@
         <v>219.5</v>
       </c>
       <c r="H18" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I18" t="n">
-        <v>208.5</v>
+        <v>210.5</v>
       </c>
       <c r="J18" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -1444,13 +1444,13 @@
         <v>285.5</v>
       </c>
       <c r="H19" t="n">
-        <v>28.80510204081634</v>
+        <v>5</v>
       </c>
       <c r="I19" t="n">
-        <v>256.6948979591837</v>
+        <v>280.5</v>
       </c>
       <c r="J19" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1485,7 +1485,7 @@
         <v>19</v>
       </c>
       <c r="D20" t="n">
-        <v>122.803</v>
+        <v>117.645</v>
       </c>
       <c r="E20" t="n">
         <v>43.091</v>
@@ -1497,19 +1497,19 @@
         <v>320</v>
       </c>
       <c r="H20" t="n">
-        <v>31.78265306122448</v>
+        <v>3.5</v>
       </c>
       <c r="I20" t="n">
-        <v>288.2173469387755</v>
+        <v>316.5</v>
       </c>
       <c r="J20" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>125.3091836734694</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M20" t="n">
         <v>47.87888888888889</v>
@@ -1644,7 +1644,7 @@
         <v>22</v>
       </c>
       <c r="D23" t="n">
-        <v>119.884</v>
+        <v>110.043</v>
       </c>
       <c r="E23" t="n">
         <v>40.775</v>
@@ -1671,16 +1671,16 @@
         <v>79.5</v>
       </c>
       <c r="M23" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N23" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O23" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P23" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q23" t="n">
         <v>-0</v>
@@ -1962,7 +1962,7 @@
         <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>68.551</v>
+        <v>68.483</v>
       </c>
       <c r="E29" t="n">
         <v>38.078</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>63.45</v>
+        <v>63.38061224489796</v>
       </c>
       <c r="L29" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M29" t="n">
         <v>42.30888888888889</v>
@@ -2121,7 +2121,7 @@
         <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>75.066</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E32" t="n">
         <v>48.821</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>63.09795918367347</v>
+        <v>72.33469387755102</v>
       </c>
       <c r="L32" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M32" t="n">
         <v>54.24555555555555</v>
@@ -2280,7 +2280,7 @@
         <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>125.853</v>
+        <v>138.408</v>
       </c>
       <c r="E35" t="n">
         <v>45.383</v>
@@ -2298,13 +2298,13 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K35" t="n">
         <v>45</v>
       </c>
       <c r="L35" t="n">
-        <v>128.4214285714286</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M35" t="n">
         <v>50.42555555555556</v>
@@ -2345,16 +2345,16 @@
         <v>4</v>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="J36" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K36" t="n">
-        <v>17.91836734693877</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
         <v>141.2326530612245</v>
@@ -2372,7 +2372,7 @@
         <v>45.38300000000001</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="37">
@@ -2398,16 +2398,16 @@
         <v>4</v>
       </c>
       <c r="H37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J37" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K37" t="n">
-        <v>20.43877551020408</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
         <v>141.9255102040816</v>
@@ -2425,7 +2425,7 @@
         <v>49.5</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="38">
@@ -2439,7 +2439,7 @@
         <v>13</v>
       </c>
       <c r="D38" t="n">
-        <v>139.087</v>
+        <v>136.236</v>
       </c>
       <c r="E38" t="n">
         <v>56.911</v>
@@ -2451,19 +2451,19 @@
         <v>4</v>
       </c>
       <c r="H38" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="J38" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K38" t="n">
-        <v>23.19081632653061</v>
+        <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>141.9255102040816</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M38" t="n">
         <v>63.23444444444445</v>
@@ -2478,7 +2478,7 @@
         <v>56.91100000000001</v>
       </c>
       <c r="Q38" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="39">
@@ -2510,10 +2510,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K39" t="n">
-        <v>20.78163265306122</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>139.0163265306122</v>
@@ -2598,7 +2598,7 @@
         <v>16</v>
       </c>
       <c r="D41" t="n">
-        <v>122.799</v>
+        <v>140.444</v>
       </c>
       <c r="E41" t="n">
         <v>41.57</v>
@@ -2610,19 +2610,19 @@
         <v>11</v>
       </c>
       <c r="H41" t="n">
-        <v>4.761224489795921</v>
+        <v>11</v>
       </c>
       <c r="I41" t="n">
-        <v>6.238775510204079</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>125.3051020408163</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M41" t="n">
         <v>46.18888888888889</v>
@@ -2637,7 +2637,7 @@
         <v>41.57</v>
       </c>
       <c r="Q41" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2663,13 +2663,13 @@
         <v>11</v>
       </c>
       <c r="H42" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2690,7 +2690,7 @@
         <v>41.57</v>
       </c>
       <c r="Q42" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="43">
@@ -2716,16 +2716,16 @@
         <v>20.5</v>
       </c>
       <c r="H43" t="n">
-        <v>20.5</v>
+        <v>5</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>15.5</v>
       </c>
       <c r="J43" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K43" t="n">
-        <v>8.305102040816337</v>
+        <v>0</v>
       </c>
       <c r="L43" t="n">
         <v>125.3091836734694</v>
@@ -2743,7 +2743,7 @@
         <v>48.767</v>
       </c>
       <c r="Q43" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="44">
@@ -2757,7 +2757,7 @@
         <v>19</v>
       </c>
       <c r="D44" t="n">
-        <v>122.803</v>
+        <v>117.645</v>
       </c>
       <c r="E44" t="n">
         <v>43.091</v>
@@ -2769,19 +2769,19 @@
         <v>28</v>
       </c>
       <c r="H44" t="n">
-        <v>28</v>
+        <v>3.5</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>24.5</v>
       </c>
       <c r="J44" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K44" t="n">
-        <v>3.78265306122448</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>125.3091836734694</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M44" t="n">
         <v>47.87888888888889</v>
@@ -2796,7 +2796,7 @@
         <v>43.09100000000001</v>
       </c>
       <c r="Q44" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="45">
@@ -2916,7 +2916,7 @@
         <v>22</v>
       </c>
       <c r="D47" t="n">
-        <v>119.884</v>
+        <v>110.043</v>
       </c>
       <c r="E47" t="n">
         <v>40.775</v>
@@ -2943,16 +2943,16 @@
         <v>79.5</v>
       </c>
       <c r="M47" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N47" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O47" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P47" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q47" t="n">
         <v>0</v>
@@ -3234,7 +3234,7 @@
         <v>4</v>
       </c>
       <c r="D53" t="n">
-        <v>68.551</v>
+        <v>68.483</v>
       </c>
       <c r="E53" t="n">
         <v>38.078</v>
@@ -3246,10 +3246,10 @@
         <v>127.5</v>
       </c>
       <c r="H53" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="I53" t="n">
-        <v>57.55</v>
+        <v>57.61938775510204</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -3258,7 +3258,7 @@
         <v>0</v>
       </c>
       <c r="L53" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M53" t="n">
         <v>42.30888888888889</v>
@@ -3393,7 +3393,7 @@
         <v>7</v>
       </c>
       <c r="D56" t="n">
-        <v>75.066</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E56" t="n">
         <v>48.821</v>
@@ -3405,10 +3405,10 @@
         <v>95.5</v>
       </c>
       <c r="H56" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="I56" t="n">
-        <v>18.90204081632653</v>
+        <v>9.665306122448982</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -3417,7 +3417,7 @@
         <v>0</v>
       </c>
       <c r="L56" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M56" t="n">
         <v>54.24555555555555</v>
@@ -3552,7 +3552,7 @@
         <v>10</v>
       </c>
       <c r="D59" t="n">
-        <v>125.853</v>
+        <v>138.408</v>
       </c>
       <c r="E59" t="n">
         <v>45.383</v>
@@ -3570,13 +3570,13 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
       </c>
       <c r="L59" t="n">
-        <v>128.4214285714286</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M59" t="n">
         <v>50.42555555555556</v>
@@ -3617,13 +3617,13 @@
         <v>32</v>
       </c>
       <c r="H60" t="n">
-        <v>21.91836734693877</v>
+        <v>0.5</v>
       </c>
       <c r="I60" t="n">
-        <v>10.08163265306123</v>
+        <v>31.5</v>
       </c>
       <c r="J60" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -3670,13 +3670,13 @@
         <v>64.5</v>
       </c>
       <c r="H61" t="n">
-        <v>24.43877551020408</v>
+        <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>40.06122448979592</v>
+        <v>63.5</v>
       </c>
       <c r="J61" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -3711,7 +3711,7 @@
         <v>13</v>
       </c>
       <c r="D62" t="n">
-        <v>139.087</v>
+        <v>136.236</v>
       </c>
       <c r="E62" t="n">
         <v>56.911</v>
@@ -3723,19 +3723,19 @@
         <v>78.5</v>
       </c>
       <c r="H62" t="n">
-        <v>27.19081632653061</v>
+        <v>1.5</v>
       </c>
       <c r="I62" t="n">
-        <v>51.30918367346939</v>
+        <v>77</v>
       </c>
       <c r="J62" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
       </c>
       <c r="L62" t="n">
-        <v>141.9255102040816</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M62" t="n">
         <v>63.23444444444445</v>
@@ -3776,13 +3776,13 @@
         <v>72.5</v>
       </c>
       <c r="H63" t="n">
-        <v>24.28163265306122</v>
+        <v>3.5</v>
       </c>
       <c r="I63" t="n">
-        <v>48.21836734693878</v>
+        <v>69</v>
       </c>
       <c r="J63" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -3870,7 +3870,7 @@
         <v>16</v>
       </c>
       <c r="D65" t="n">
-        <v>122.799</v>
+        <v>140.444</v>
       </c>
       <c r="E65" t="n">
         <v>41.57</v>
@@ -3882,19 +3882,19 @@
         <v>69.5</v>
       </c>
       <c r="H65" t="n">
-        <v>4.761224489795921</v>
+        <v>11</v>
       </c>
       <c r="I65" t="n">
-        <v>64.73877551020408</v>
+        <v>58.5</v>
       </c>
       <c r="J65" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
       </c>
       <c r="L65" t="n">
-        <v>125.3051020408163</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M65" t="n">
         <v>46.18888888888889</v>
@@ -3935,13 +3935,13 @@
         <v>72</v>
       </c>
       <c r="H66" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I66" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J66" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3988,13 +3988,13 @@
         <v>74.5</v>
       </c>
       <c r="H67" t="n">
-        <v>28.80510204081634</v>
+        <v>5</v>
       </c>
       <c r="I67" t="n">
-        <v>45.69489795918366</v>
+        <v>69.5</v>
       </c>
       <c r="J67" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -4029,7 +4029,7 @@
         <v>19</v>
       </c>
       <c r="D68" t="n">
-        <v>122.803</v>
+        <v>117.645</v>
       </c>
       <c r="E68" t="n">
         <v>43.091</v>
@@ -4041,19 +4041,19 @@
         <v>81.5</v>
       </c>
       <c r="H68" t="n">
-        <v>31.78265306122448</v>
+        <v>3.5</v>
       </c>
       <c r="I68" t="n">
-        <v>49.71734693877552</v>
+        <v>78</v>
       </c>
       <c r="J68" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
       </c>
       <c r="L68" t="n">
-        <v>125.3091836734694</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M68" t="n">
         <v>47.87888888888889</v>
@@ -4188,7 +4188,7 @@
         <v>22</v>
       </c>
       <c r="D71" t="n">
-        <v>119.884</v>
+        <v>110.043</v>
       </c>
       <c r="E71" t="n">
         <v>40.775</v>
@@ -4215,16 +4215,16 @@
         <v>79.5</v>
       </c>
       <c r="M71" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N71" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666668</v>
       </c>
       <c r="O71" t="n">
-        <v>9.031728395061723</v>
+        <v>17.53629629629629</v>
       </c>
       <c r="P71" t="n">
-        <v>8.12855555555555</v>
+        <v>15.78266666666666</v>
       </c>
       <c r="Q71" t="n">
         <v>0</v>
@@ -4506,7 +4506,7 @@
         <v>4</v>
       </c>
       <c r="D77" t="n">
-        <v>68.551</v>
+        <v>68.483</v>
       </c>
       <c r="E77" t="n">
         <v>38.078</v>
@@ -4518,10 +4518,10 @@
         <v>143</v>
       </c>
       <c r="H77" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="I77" t="n">
-        <v>73.05</v>
+        <v>73.11938775510204</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
@@ -4530,7 +4530,7 @@
         <v>0</v>
       </c>
       <c r="L77" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M77" t="n">
         <v>42.30888888888889</v>
@@ -4665,7 +4665,7 @@
         <v>7</v>
       </c>
       <c r="D80" t="n">
-        <v>75.066</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E80" t="n">
         <v>48.821</v>
@@ -4677,10 +4677,10 @@
         <v>139</v>
       </c>
       <c r="H80" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="I80" t="n">
-        <v>62.40204081632653</v>
+        <v>53.16530612244898</v>
       </c>
       <c r="J80" t="n">
         <v>0</v>
@@ -4689,7 +4689,7 @@
         <v>0</v>
       </c>
       <c r="L80" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M80" t="n">
         <v>54.24555555555555</v>
@@ -4824,7 +4824,7 @@
         <v>10</v>
       </c>
       <c r="D83" t="n">
-        <v>125.853</v>
+        <v>138.408</v>
       </c>
       <c r="E83" t="n">
         <v>45.383</v>
@@ -4842,13 +4842,13 @@
         <v>89</v>
       </c>
       <c r="J83" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
       </c>
       <c r="L83" t="n">
-        <v>128.4214285714286</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M83" t="n">
         <v>50.42555555555556</v>
@@ -4889,13 +4889,13 @@
         <v>142.5</v>
       </c>
       <c r="H84" t="n">
-        <v>21.91836734693877</v>
+        <v>0.5</v>
       </c>
       <c r="I84" t="n">
-        <v>120.5816326530612</v>
+        <v>142</v>
       </c>
       <c r="J84" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -4942,13 +4942,13 @@
         <v>139</v>
       </c>
       <c r="H85" t="n">
-        <v>24.43877551020408</v>
+        <v>1</v>
       </c>
       <c r="I85" t="n">
-        <v>114.5612244897959</v>
+        <v>138</v>
       </c>
       <c r="J85" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -4983,7 +4983,7 @@
         <v>13</v>
       </c>
       <c r="D86" t="n">
-        <v>139.087</v>
+        <v>136.236</v>
       </c>
       <c r="E86" t="n">
         <v>56.911</v>
@@ -4995,19 +4995,19 @@
         <v>128</v>
       </c>
       <c r="H86" t="n">
-        <v>27.19081632653061</v>
+        <v>1.5</v>
       </c>
       <c r="I86" t="n">
-        <v>100.8091836734694</v>
+        <v>126.5</v>
       </c>
       <c r="J86" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>141.9255102040816</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M86" t="n">
         <v>63.23444444444445</v>
@@ -5048,13 +5048,13 @@
         <v>118.5</v>
       </c>
       <c r="H87" t="n">
-        <v>24.28163265306122</v>
+        <v>3.5</v>
       </c>
       <c r="I87" t="n">
-        <v>94.21836734693878</v>
+        <v>115</v>
       </c>
       <c r="J87" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -5142,7 +5142,7 @@
         <v>16</v>
       </c>
       <c r="D89" t="n">
-        <v>122.799</v>
+        <v>140.444</v>
       </c>
       <c r="E89" t="n">
         <v>41.57</v>
@@ -5154,19 +5154,19 @@
         <v>152.5</v>
       </c>
       <c r="H89" t="n">
-        <v>4.761224489795921</v>
+        <v>11</v>
       </c>
       <c r="I89" t="n">
-        <v>147.7387755102041</v>
+        <v>141.5</v>
       </c>
       <c r="J89" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K89" t="n">
         <v>0</v>
       </c>
       <c r="L89" t="n">
-        <v>125.3051020408163</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M89" t="n">
         <v>46.18888888888889</v>
@@ -5207,13 +5207,13 @@
         <v>170.5</v>
       </c>
       <c r="H90" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I90" t="n">
-        <v>159.5</v>
+        <v>161.5</v>
       </c>
       <c r="J90" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K90" t="n">
         <v>0</v>
@@ -5260,13 +5260,13 @@
         <v>174</v>
       </c>
       <c r="H91" t="n">
-        <v>28.80510204081634</v>
+        <v>5</v>
       </c>
       <c r="I91" t="n">
-        <v>145.1948979591837</v>
+        <v>169</v>
       </c>
       <c r="J91" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K91" t="n">
         <v>0</v>
@@ -5301,7 +5301,7 @@
         <v>19</v>
       </c>
       <c r="D92" t="n">
-        <v>122.803</v>
+        <v>117.645</v>
       </c>
       <c r="E92" t="n">
         <v>43.091</v>
@@ -5313,19 +5313,19 @@
         <v>162.5</v>
       </c>
       <c r="H92" t="n">
-        <v>31.78265306122448</v>
+        <v>3.5</v>
       </c>
       <c r="I92" t="n">
-        <v>130.7173469387755</v>
+        <v>159</v>
       </c>
       <c r="J92" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K92" t="n">
         <v>0</v>
       </c>
       <c r="L92" t="n">
-        <v>125.3091836734694</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M92" t="n">
         <v>47.87888888888889</v>
@@ -5460,7 +5460,7 @@
         <v>22</v>
       </c>
       <c r="D95" t="n">
-        <v>119.884</v>
+        <v>110.043</v>
       </c>
       <c r="E95" t="n">
         <v>40.775</v>
@@ -5487,16 +5487,16 @@
         <v>79.5</v>
       </c>
       <c r="M95" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N95" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O95" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P95" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q95" t="n">
         <v>-0</v>
@@ -5778,7 +5778,7 @@
         <v>4</v>
       </c>
       <c r="D101" t="n">
-        <v>68.551</v>
+        <v>68.483</v>
       </c>
       <c r="E101" t="n">
         <v>38.078</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="K101" t="n">
-        <v>59.45</v>
+        <v>59.38061224489796</v>
       </c>
       <c r="L101" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M101" t="n">
         <v>42.30888888888889</v>
@@ -5937,7 +5937,7 @@
         <v>7</v>
       </c>
       <c r="D104" t="n">
-        <v>75.066</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E104" t="n">
         <v>48.821</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="K104" t="n">
-        <v>53.09795918367347</v>
+        <v>62.33469387755102</v>
       </c>
       <c r="L104" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M104" t="n">
         <v>54.24555555555555</v>
@@ -6096,7 +6096,7 @@
         <v>10</v>
       </c>
       <c r="D107" t="n">
-        <v>125.853</v>
+        <v>138.408</v>
       </c>
       <c r="E107" t="n">
         <v>45.383</v>
@@ -6114,13 +6114,13 @@
         <v>0</v>
       </c>
       <c r="J107" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K107" t="n">
         <v>43</v>
       </c>
       <c r="L107" t="n">
-        <v>128.4214285714286</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M107" t="n">
         <v>50.42555555555556</v>
@@ -6161,16 +6161,16 @@
         <v>4</v>
       </c>
       <c r="H108" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="I108" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="J108" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K108" t="n">
-        <v>17.91836734693877</v>
+        <v>0</v>
       </c>
       <c r="L108" t="n">
         <v>141.2326530612245</v>
@@ -6214,16 +6214,16 @@
         <v>3</v>
       </c>
       <c r="H109" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I109" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J109" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K109" t="n">
-        <v>21.43877551020408</v>
+        <v>0</v>
       </c>
       <c r="L109" t="n">
         <v>141.9255102040816</v>
@@ -6241,7 +6241,7 @@
         <v>49.5</v>
       </c>
       <c r="Q109" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="110">
@@ -6255,7 +6255,7 @@
         <v>13</v>
       </c>
       <c r="D110" t="n">
-        <v>139.087</v>
+        <v>136.236</v>
       </c>
       <c r="E110" t="n">
         <v>56.911</v>
@@ -6267,19 +6267,19 @@
         <v>2.5</v>
       </c>
       <c r="H110" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="I110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J110" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K110" t="n">
-        <v>24.69081632653061</v>
+        <v>0</v>
       </c>
       <c r="L110" t="n">
-        <v>141.9255102040816</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M110" t="n">
         <v>63.23444444444445</v>
@@ -6326,10 +6326,10 @@
         <v>0</v>
       </c>
       <c r="J111" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K111" t="n">
-        <v>22.28163265306122</v>
+        <v>1.5</v>
       </c>
       <c r="L111" t="n">
         <v>139.0163265306122</v>
@@ -6414,7 +6414,7 @@
         <v>16</v>
       </c>
       <c r="D113" t="n">
-        <v>122.799</v>
+        <v>140.444</v>
       </c>
       <c r="E113" t="n">
         <v>41.57</v>
@@ -6426,19 +6426,19 @@
         <v>6</v>
       </c>
       <c r="H113" t="n">
-        <v>4.761224489795921</v>
+        <v>6</v>
       </c>
       <c r="I113" t="n">
-        <v>1.238775510204079</v>
+        <v>0</v>
       </c>
       <c r="J113" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K113" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L113" t="n">
-        <v>125.3051020408163</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M113" t="n">
         <v>46.18888888888889</v>
@@ -6479,13 +6479,13 @@
         <v>12.5</v>
       </c>
       <c r="H114" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I114" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="J114" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -6532,16 +6532,16 @@
         <v>17</v>
       </c>
       <c r="H115" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="I115" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J115" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K115" t="n">
-        <v>11.80510204081634</v>
+        <v>0</v>
       </c>
       <c r="L115" t="n">
         <v>125.3091836734694</v>
@@ -6573,7 +6573,7 @@
         <v>19</v>
       </c>
       <c r="D116" t="n">
-        <v>122.803</v>
+        <v>117.645</v>
       </c>
       <c r="E116" t="n">
         <v>43.091</v>
@@ -6585,19 +6585,19 @@
         <v>18.5</v>
       </c>
       <c r="H116" t="n">
-        <v>18.5</v>
+        <v>3.5</v>
       </c>
       <c r="I116" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J116" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K116" t="n">
-        <v>13.28265306122448</v>
+        <v>0</v>
       </c>
       <c r="L116" t="n">
-        <v>125.3091836734694</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M116" t="n">
         <v>47.87888888888889</v>
@@ -6732,7 +6732,7 @@
         <v>22</v>
       </c>
       <c r="D119" t="n">
-        <v>119.884</v>
+        <v>110.043</v>
       </c>
       <c r="E119" t="n">
         <v>40.775</v>
@@ -6759,16 +6759,16 @@
         <v>79.5</v>
       </c>
       <c r="M119" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N119" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O119" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P119" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q119" t="n">
         <v>0</v>
@@ -7050,7 +7050,7 @@
         <v>4</v>
       </c>
       <c r="D125" t="n">
-        <v>68.551</v>
+        <v>68.483</v>
       </c>
       <c r="E125" t="n">
         <v>38.078</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="K125" t="n">
-        <v>48.95</v>
+        <v>48.88061224489796</v>
       </c>
       <c r="L125" t="n">
-        <v>69.95</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M125" t="n">
         <v>42.30888888888889</v>
@@ -7209,7 +7209,7 @@
         <v>7</v>
       </c>
       <c r="D128" t="n">
-        <v>75.066</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E128" t="n">
         <v>48.821</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="K128" t="n">
-        <v>49.09795918367347</v>
+        <v>58.33469387755102</v>
       </c>
       <c r="L128" t="n">
-        <v>76.59795918367347</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M128" t="n">
         <v>54.24555555555555</v>
@@ -7368,7 +7368,7 @@
         <v>10</v>
       </c>
       <c r="D131" t="n">
-        <v>125.853</v>
+        <v>138.408</v>
       </c>
       <c r="E131" t="n">
         <v>45.383</v>
@@ -7386,13 +7386,13 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K131" t="n">
         <v>48</v>
       </c>
       <c r="L131" t="n">
-        <v>128.4214285714286</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M131" t="n">
         <v>50.42555555555556</v>
@@ -7439,10 +7439,10 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K132" t="n">
-        <v>21.41836734693877</v>
+        <v>0</v>
       </c>
       <c r="L132" t="n">
         <v>141.2326530612245</v>
@@ -7460,7 +7460,7 @@
         <v>45.38300000000001</v>
       </c>
       <c r="Q132" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="133">
@@ -7492,10 +7492,10 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K133" t="n">
-        <v>23.43877551020408</v>
+        <v>-0</v>
       </c>
       <c r="L133" t="n">
         <v>141.9255102040816</v>
@@ -7527,7 +7527,7 @@
         <v>13</v>
       </c>
       <c r="D134" t="n">
-        <v>139.087</v>
+        <v>136.236</v>
       </c>
       <c r="E134" t="n">
         <v>56.911</v>
@@ -7545,13 +7545,13 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K134" t="n">
-        <v>25.69081632653061</v>
+        <v>-0</v>
       </c>
       <c r="L134" t="n">
-        <v>141.9255102040816</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M134" t="n">
         <v>63.23444444444445</v>
@@ -7598,10 +7598,10 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K135" t="n">
-        <v>21.78163265306122</v>
+        <v>1</v>
       </c>
       <c r="L135" t="n">
         <v>139.0163265306122</v>
@@ -7686,7 +7686,7 @@
         <v>16</v>
       </c>
       <c r="D137" t="n">
-        <v>122.799</v>
+        <v>140.444</v>
       </c>
       <c r="E137" t="n">
         <v>41.57</v>
@@ -7698,19 +7698,19 @@
         <v>10.5</v>
       </c>
       <c r="H137" t="n">
-        <v>4.761224489795921</v>
+        <v>10.5</v>
       </c>
       <c r="I137" t="n">
-        <v>5.738775510204079</v>
+        <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K137" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L137" t="n">
-        <v>125.3051020408163</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M137" t="n">
         <v>46.18888888888889</v>
@@ -7725,7 +7725,7 @@
         <v>41.57</v>
       </c>
       <c r="Q137" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -7751,16 +7751,16 @@
         <v>10.5</v>
       </c>
       <c r="H138" t="n">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="I138" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="J138" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K138" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L138" t="n">
         <v>143.3102040816326</v>
@@ -7778,7 +7778,7 @@
         <v>41.57</v>
       </c>
       <c r="Q138" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="139">
@@ -7804,16 +7804,16 @@
         <v>14.5</v>
       </c>
       <c r="H139" t="n">
-        <v>14.5</v>
+        <v>5</v>
       </c>
       <c r="I139" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J139" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K139" t="n">
-        <v>14.30510204081634</v>
+        <v>0</v>
       </c>
       <c r="L139" t="n">
         <v>125.3091836734694</v>
@@ -7831,7 +7831,7 @@
         <v>48.767</v>
       </c>
       <c r="Q139" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="140">
@@ -7845,7 +7845,7 @@
         <v>19</v>
       </c>
       <c r="D140" t="n">
-        <v>122.803</v>
+        <v>117.645</v>
       </c>
       <c r="E140" t="n">
         <v>43.091</v>
@@ -7857,19 +7857,19 @@
         <v>30</v>
       </c>
       <c r="H140" t="n">
-        <v>30</v>
+        <v>3.5</v>
       </c>
       <c r="I140" t="n">
-        <v>0</v>
+        <v>26.5</v>
       </c>
       <c r="J140" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K140" t="n">
-        <v>1.78265306122448</v>
+        <v>0</v>
       </c>
       <c r="L140" t="n">
-        <v>125.3091836734694</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M140" t="n">
         <v>47.87888888888889</v>
@@ -7884,7 +7884,7 @@
         <v>43.09100000000001</v>
       </c>
       <c r="Q140" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="141">
@@ -8004,7 +8004,7 @@
         <v>22</v>
       </c>
       <c r="D143" t="n">
-        <v>119.884</v>
+        <v>110.043</v>
       </c>
       <c r="E143" t="n">
         <v>40.775</v>
@@ -8031,16 +8031,16 @@
         <v>79.5</v>
       </c>
       <c r="M143" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N143" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O143" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P143" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q143" t="n">
         <v>0</v>
@@ -8652,16 +8652,16 @@
         <v>56</v>
       </c>
       <c r="H155" t="n">
-        <v>56</v>
+        <v>50.5</v>
       </c>
       <c r="I155" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="J155" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K155" t="n">
-        <v>7.311224489795904</v>
+        <v>0</v>
       </c>
       <c r="L155" t="n">
         <v>141.2326530612245</v>
@@ -8679,7 +8679,7 @@
         <v>45.38300000000001</v>
       </c>
       <c r="Q155" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="156">
@@ -8705,13 +8705,13 @@
         <v>63.5</v>
       </c>
       <c r="H156" t="n">
-        <v>21.91836734693877</v>
+        <v>0.5</v>
       </c>
       <c r="I156" t="n">
-        <v>41.58163265306123</v>
+        <v>63</v>
       </c>
       <c r="J156" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K156" t="n">
         <v>0</v>
@@ -8758,13 +8758,13 @@
         <v>67</v>
       </c>
       <c r="H157" t="n">
-        <v>24.43877551020408</v>
+        <v>1</v>
       </c>
       <c r="I157" t="n">
-        <v>42.56122448979592</v>
+        <v>66</v>
       </c>
       <c r="J157" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K157" t="n">
         <v>0</v>
@@ -8811,13 +8811,13 @@
         <v>68</v>
       </c>
       <c r="H158" t="n">
-        <v>24.28163265306122</v>
+        <v>1.5</v>
       </c>
       <c r="I158" t="n">
-        <v>43.71836734693878</v>
+        <v>66.5</v>
       </c>
       <c r="J158" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K158" t="n">
         <v>0</v>
@@ -8864,13 +8864,13 @@
         <v>70</v>
       </c>
       <c r="H159" t="n">
-        <v>24.28163265306122</v>
+        <v>3.5</v>
       </c>
       <c r="I159" t="n">
-        <v>45.71836734693878</v>
+        <v>66.5</v>
       </c>
       <c r="J159" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K159" t="n">
         <v>0</v>
@@ -8970,13 +8970,13 @@
         <v>67.5</v>
       </c>
       <c r="H161" t="n">
-        <v>22.76632653061222</v>
+        <v>11</v>
       </c>
       <c r="I161" t="n">
-        <v>44.73367346938778</v>
+        <v>56.5</v>
       </c>
       <c r="J161" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K161" t="n">
         <v>0</v>
@@ -9023,13 +9023,13 @@
         <v>62.5</v>
       </c>
       <c r="H162" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I162" t="n">
-        <v>51.5</v>
+        <v>53.5</v>
       </c>
       <c r="J162" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K162" t="n">
         <v>0</v>
@@ -9076,13 +9076,13 @@
         <v>57.5</v>
       </c>
       <c r="H163" t="n">
-        <v>28.80510204081634</v>
+        <v>5</v>
       </c>
       <c r="I163" t="n">
-        <v>28.69489795918366</v>
+        <v>52.5</v>
       </c>
       <c r="J163" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K163" t="n">
         <v>0</v>
@@ -9129,13 +9129,13 @@
         <v>56</v>
       </c>
       <c r="H164" t="n">
-        <v>26.51938775510203</v>
+        <v>3.5</v>
       </c>
       <c r="I164" t="n">
-        <v>29.48061224489797</v>
+        <v>52.5</v>
       </c>
       <c r="J164" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K164" t="n">
         <v>0</v>
@@ -9297,22 +9297,22 @@
         <v>0</v>
       </c>
       <c r="K167" t="n">
-        <v>7.958163265306126</v>
+        <v>18</v>
       </c>
       <c r="L167" t="n">
-        <v>69.45816326530613</v>
+        <v>79.5</v>
       </c>
       <c r="M167" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N167" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O167" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P167" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q167" t="n">
         <v>0</v>
@@ -9924,13 +9924,13 @@
         <v>246.5</v>
       </c>
       <c r="H179" t="n">
-        <v>63.3112244897959</v>
+        <v>50.5</v>
       </c>
       <c r="I179" t="n">
-        <v>183.1887755102041</v>
+        <v>196</v>
       </c>
       <c r="J179" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K179" t="n">
         <v>0</v>
@@ -9977,13 +9977,13 @@
         <v>266.5</v>
       </c>
       <c r="H180" t="n">
-        <v>21.91836734693877</v>
+        <v>0.5</v>
       </c>
       <c r="I180" t="n">
-        <v>244.5816326530612</v>
+        <v>266</v>
       </c>
       <c r="J180" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K180" t="n">
         <v>0</v>
@@ -10030,13 +10030,13 @@
         <v>293.5</v>
       </c>
       <c r="H181" t="n">
-        <v>24.43877551020408</v>
+        <v>1</v>
       </c>
       <c r="I181" t="n">
-        <v>269.0612244897959</v>
+        <v>292.5</v>
       </c>
       <c r="J181" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K181" t="n">
         <v>0</v>
@@ -10083,13 +10083,13 @@
         <v>306</v>
       </c>
       <c r="H182" t="n">
-        <v>24.28163265306122</v>
+        <v>1.5</v>
       </c>
       <c r="I182" t="n">
-        <v>281.7183673469387</v>
+        <v>304.5</v>
       </c>
       <c r="J182" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K182" t="n">
         <v>0</v>
@@ -10136,13 +10136,13 @@
         <v>293.5</v>
       </c>
       <c r="H183" t="n">
-        <v>24.28163265306122</v>
+        <v>3.5</v>
       </c>
       <c r="I183" t="n">
-        <v>269.2183673469387</v>
+        <v>290</v>
       </c>
       <c r="J183" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K183" t="n">
         <v>0</v>
@@ -10242,13 +10242,13 @@
         <v>280</v>
       </c>
       <c r="H185" t="n">
-        <v>22.76632653061222</v>
+        <v>11</v>
       </c>
       <c r="I185" t="n">
-        <v>257.2336734693878</v>
+        <v>269</v>
       </c>
       <c r="J185" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K185" t="n">
         <v>0</v>
@@ -10295,13 +10295,13 @@
         <v>222</v>
       </c>
       <c r="H186" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I186" t="n">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="J186" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K186" t="n">
         <v>0</v>
@@ -10348,13 +10348,13 @@
         <v>155.5</v>
       </c>
       <c r="H187" t="n">
-        <v>28.80510204081634</v>
+        <v>5</v>
       </c>
       <c r="I187" t="n">
-        <v>126.6948979591837</v>
+        <v>150.5</v>
       </c>
       <c r="J187" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K187" t="n">
         <v>0</v>
@@ -10401,13 +10401,13 @@
         <v>133</v>
       </c>
       <c r="H188" t="n">
-        <v>26.51938775510203</v>
+        <v>3.5</v>
       </c>
       <c r="I188" t="n">
-        <v>106.480612244898</v>
+        <v>129.5</v>
       </c>
       <c r="J188" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K188" t="n">
         <v>0</v>
@@ -10560,10 +10560,10 @@
         <v>155</v>
       </c>
       <c r="H191" t="n">
-        <v>69.45816326530613</v>
+        <v>79.5</v>
       </c>
       <c r="I191" t="n">
-        <v>85.54183673469387</v>
+        <v>75.5</v>
       </c>
       <c r="J191" t="n">
         <v>0</v>
@@ -10572,19 +10572,19 @@
         <v>0</v>
       </c>
       <c r="L191" t="n">
-        <v>69.45816326530613</v>
+        <v>79.5</v>
       </c>
       <c r="M191" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N191" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O191" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P191" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q191" t="n">
         <v>-0</v>
@@ -11202,10 +11202,10 @@
         <v>0</v>
       </c>
       <c r="J203" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K203" t="n">
-        <v>34.8112244897959</v>
+        <v>22</v>
       </c>
       <c r="L203" t="n">
         <v>141.2326530612245</v>
@@ -11249,13 +11249,13 @@
         <v>27</v>
       </c>
       <c r="H204" t="n">
-        <v>21.91836734693877</v>
+        <v>0.5</v>
       </c>
       <c r="I204" t="n">
-        <v>5.081632653061234</v>
+        <v>26.5</v>
       </c>
       <c r="J204" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K204" t="n">
         <v>0</v>
@@ -11302,13 +11302,13 @@
         <v>29.5</v>
       </c>
       <c r="H205" t="n">
-        <v>24.43877551020408</v>
+        <v>1</v>
       </c>
       <c r="I205" t="n">
-        <v>5.061224489795919</v>
+        <v>28.5</v>
       </c>
       <c r="J205" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K205" t="n">
         <v>0</v>
@@ -11355,13 +11355,13 @@
         <v>31.5</v>
       </c>
       <c r="H206" t="n">
-        <v>24.28163265306122</v>
+        <v>1.5</v>
       </c>
       <c r="I206" t="n">
-        <v>7.218367346938777</v>
+        <v>30</v>
       </c>
       <c r="J206" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K206" t="n">
         <v>0</v>
@@ -11408,13 +11408,13 @@
         <v>36</v>
       </c>
       <c r="H207" t="n">
-        <v>24.28163265306122</v>
+        <v>3.5</v>
       </c>
       <c r="I207" t="n">
-        <v>11.71836734693878</v>
+        <v>32.5</v>
       </c>
       <c r="J207" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K207" t="n">
         <v>0</v>
@@ -11514,13 +11514,13 @@
         <v>45</v>
       </c>
       <c r="H209" t="n">
-        <v>22.76632653061222</v>
+        <v>11</v>
       </c>
       <c r="I209" t="n">
-        <v>22.23367346938778</v>
+        <v>34</v>
       </c>
       <c r="J209" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K209" t="n">
         <v>0</v>
@@ -11567,13 +11567,13 @@
         <v>38.5</v>
       </c>
       <c r="H210" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I210" t="n">
-        <v>27.5</v>
+        <v>29.5</v>
       </c>
       <c r="J210" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K210" t="n">
         <v>0</v>
@@ -11620,13 +11620,13 @@
         <v>42.5</v>
       </c>
       <c r="H211" t="n">
-        <v>28.80510204081634</v>
+        <v>5</v>
       </c>
       <c r="I211" t="n">
-        <v>13.69489795918366</v>
+        <v>37.5</v>
       </c>
       <c r="J211" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K211" t="n">
         <v>0</v>
@@ -11673,13 +11673,13 @@
         <v>50.5</v>
       </c>
       <c r="H212" t="n">
-        <v>26.51938775510203</v>
+        <v>3.5</v>
       </c>
       <c r="I212" t="n">
-        <v>23.98061224489797</v>
+        <v>47</v>
       </c>
       <c r="J212" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K212" t="n">
         <v>0</v>
@@ -11841,22 +11841,22 @@
         <v>0</v>
       </c>
       <c r="K215" t="n">
-        <v>62.95816326530613</v>
+        <v>73</v>
       </c>
       <c r="L215" t="n">
-        <v>69.45816326530613</v>
+        <v>79.5</v>
       </c>
       <c r="M215" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N215" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O215" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P215" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q215" t="n">
         <v>0</v>
@@ -12474,10 +12474,10 @@
         <v>0</v>
       </c>
       <c r="J227" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K227" t="n">
-        <v>63.3112244897959</v>
+        <v>50.5</v>
       </c>
       <c r="L227" t="n">
         <v>141.2326530612245</v>
@@ -12527,10 +12527,10 @@
         <v>0</v>
       </c>
       <c r="J228" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K228" t="n">
-        <v>21.91836734693877</v>
+        <v>0.5</v>
       </c>
       <c r="L228" t="n">
         <v>141.2326530612245</v>
@@ -12580,10 +12580,10 @@
         <v>0</v>
       </c>
       <c r="J229" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K229" t="n">
-        <v>23.93877551020408</v>
+        <v>0.5</v>
       </c>
       <c r="L229" t="n">
         <v>141.9255102040816</v>
@@ -12627,16 +12627,16 @@
         <v>6.5</v>
       </c>
       <c r="H230" t="n">
-        <v>6.5</v>
+        <v>1.5</v>
       </c>
       <c r="I230" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J230" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K230" t="n">
-        <v>17.78163265306122</v>
+        <v>0</v>
       </c>
       <c r="L230" t="n">
         <v>139.0163265306122</v>
@@ -12654,7 +12654,7 @@
         <v>56.91100000000001</v>
       </c>
       <c r="Q230" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="231">
@@ -12680,16 +12680,16 @@
         <v>24</v>
       </c>
       <c r="H231" t="n">
-        <v>24</v>
+        <v>3.5</v>
       </c>
       <c r="I231" t="n">
-        <v>0</v>
+        <v>20.5</v>
       </c>
       <c r="J231" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K231" t="n">
-        <v>0.281632653061223</v>
+        <v>0</v>
       </c>
       <c r="L231" t="n">
         <v>139.0163265306122</v>
@@ -12707,7 +12707,7 @@
         <v>56.91100000000001</v>
       </c>
       <c r="Q231" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="232">
@@ -12786,13 +12786,13 @@
         <v>40</v>
       </c>
       <c r="H233" t="n">
-        <v>22.76632653061222</v>
+        <v>11</v>
       </c>
       <c r="I233" t="n">
-        <v>17.23367346938778</v>
+        <v>29</v>
       </c>
       <c r="J233" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K233" t="n">
         <v>0</v>
@@ -12839,13 +12839,13 @@
         <v>49.5</v>
       </c>
       <c r="H234" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I234" t="n">
-        <v>38.5</v>
+        <v>40.5</v>
       </c>
       <c r="J234" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K234" t="n">
         <v>0</v>
@@ -12892,13 +12892,13 @@
         <v>61</v>
       </c>
       <c r="H235" t="n">
-        <v>28.80510204081634</v>
+        <v>5</v>
       </c>
       <c r="I235" t="n">
-        <v>32.19489795918366</v>
+        <v>56</v>
       </c>
       <c r="J235" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K235" t="n">
         <v>0</v>
@@ -12945,13 +12945,13 @@
         <v>64</v>
       </c>
       <c r="H236" t="n">
-        <v>26.51938775510203</v>
+        <v>3.5</v>
       </c>
       <c r="I236" t="n">
-        <v>37.48061224489797</v>
+        <v>60.5</v>
       </c>
       <c r="J236" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K236" t="n">
         <v>0</v>
@@ -13113,22 +13113,22 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>60.95816326530613</v>
+        <v>71</v>
       </c>
       <c r="L239" t="n">
-        <v>69.45816326530613</v>
+        <v>79.5</v>
       </c>
       <c r="M239" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N239" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O239" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P239" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q239" t="n">
         <v>0</v>
@@ -13251,7 +13251,7 @@
         <v>1</v>
       </c>
       <c r="D242" t="n">
-        <v>67.804</v>
+        <v>68.551</v>
       </c>
       <c r="E242" t="n">
         <v>35.363</v>
@@ -13272,10 +13272,10 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>56.18775510204082</v>
+        <v>56.95</v>
       </c>
       <c r="L242" t="n">
-        <v>69.18775510204082</v>
+        <v>69.95</v>
       </c>
       <c r="M242" t="n">
         <v>39.29222222222222</v>
@@ -13304,7 +13304,7 @@
         <v>2</v>
       </c>
       <c r="D243" t="n">
-        <v>67.804</v>
+        <v>68.551</v>
       </c>
       <c r="E243" t="n">
         <v>35.363</v>
@@ -13325,10 +13325,10 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
-        <v>56.68775510204082</v>
+        <v>57.45</v>
       </c>
       <c r="L243" t="n">
-        <v>69.18775510204082</v>
+        <v>69.95</v>
       </c>
       <c r="M243" t="n">
         <v>39.29222222222222</v>
@@ -13357,7 +13357,7 @@
         <v>3</v>
       </c>
       <c r="D244" t="n">
-        <v>67.804</v>
+        <v>68.551</v>
       </c>
       <c r="E244" t="n">
         <v>35.363</v>
@@ -13378,10 +13378,10 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
-        <v>56.18775510204082</v>
+        <v>56.95</v>
       </c>
       <c r="L244" t="n">
-        <v>69.18775510204082</v>
+        <v>69.95</v>
       </c>
       <c r="M244" t="n">
         <v>39.29222222222222</v>
@@ -13410,7 +13410,7 @@
         <v>4</v>
       </c>
       <c r="D245" t="n">
-        <v>67.804</v>
+        <v>68.483</v>
       </c>
       <c r="E245" t="n">
         <v>38.078</v>
@@ -13431,10 +13431,10 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>52.18775510204082</v>
+        <v>52.88061224489796</v>
       </c>
       <c r="L245" t="n">
-        <v>69.18775510204082</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M245" t="n">
         <v>42.30888888888889</v>
@@ -13463,7 +13463,7 @@
         <v>5</v>
       </c>
       <c r="D246" t="n">
-        <v>67.804</v>
+        <v>68.483</v>
       </c>
       <c r="E246" t="n">
         <v>38.078</v>
@@ -13484,10 +13484,10 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
-        <v>47.18775510204082</v>
+        <v>47.88061224489796</v>
       </c>
       <c r="L246" t="n">
-        <v>69.18775510204082</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M246" t="n">
         <v>42.30888888888889</v>
@@ -13516,7 +13516,7 @@
         <v>6</v>
       </c>
       <c r="D247" t="n">
-        <v>75.039</v>
+        <v>75.066</v>
       </c>
       <c r="E247" t="n">
         <v>38.078</v>
@@ -13537,10 +13537,10 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>60.57040816326531</v>
+        <v>60.59795918367347</v>
       </c>
       <c r="L247" t="n">
-        <v>76.57040816326531</v>
+        <v>76.59795918367347</v>
       </c>
       <c r="M247" t="n">
         <v>42.30888888888889</v>
@@ -13569,7 +13569,7 @@
         <v>7</v>
       </c>
       <c r="D248" t="n">
-        <v>78.58799999999999</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E248" t="n">
         <v>48.821</v>
@@ -13590,10 +13590,10 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>75.19183673469388</v>
+        <v>80.83469387755102</v>
       </c>
       <c r="L248" t="n">
-        <v>80.19183673469388</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M248" t="n">
         <v>54.24555555555555</v>
@@ -13622,7 +13622,7 @@
         <v>8</v>
       </c>
       <c r="D249" t="n">
-        <v>78.58799999999999</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E249" t="n">
         <v>48.821</v>
@@ -13643,10 +13643,10 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>79.19183673469388</v>
+        <v>84.83469387755102</v>
       </c>
       <c r="L249" t="n">
-        <v>80.19183673469388</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M249" t="n">
         <v>54.24555555555555</v>
@@ -13675,7 +13675,7 @@
         <v>9</v>
       </c>
       <c r="D250" t="n">
-        <v>118.618</v>
+        <v>125.853</v>
       </c>
       <c r="E250" t="n">
         <v>61.411</v>
@@ -13696,10 +13696,10 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>120.5387755102041</v>
+        <v>127.9214285714286</v>
       </c>
       <c r="L250" t="n">
-        <v>121.0387755102041</v>
+        <v>128.4214285714286</v>
       </c>
       <c r="M250" t="n">
         <v>68.23444444444445</v>
@@ -13728,7 +13728,7 @@
         <v>10</v>
       </c>
       <c r="D251" t="n">
-        <v>116.928</v>
+        <v>138.408</v>
       </c>
       <c r="E251" t="n">
         <v>45.383</v>
@@ -13746,13 +13746,13 @@
         <v>0</v>
       </c>
       <c r="J251" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K251" t="n">
-        <v>40.39285714285714</v>
+        <v>49.5</v>
       </c>
       <c r="L251" t="n">
-        <v>119.3142857142857</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M251" t="n">
         <v>50.42555555555556</v>
@@ -13781,7 +13781,7 @@
         <v>11</v>
       </c>
       <c r="D252" t="n">
-        <v>116.928</v>
+        <v>138.408</v>
       </c>
       <c r="E252" t="n">
         <v>45.383</v>
@@ -13793,19 +13793,19 @@
         <v>2</v>
       </c>
       <c r="H252" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I252" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J252" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K252" t="n">
         <v>0</v>
       </c>
       <c r="L252" t="n">
-        <v>119.3142857142857</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M252" t="n">
         <v>50.42555555555556</v>
@@ -13834,7 +13834,7 @@
         <v>12</v>
       </c>
       <c r="D253" t="n">
-        <v>115.137</v>
+        <v>139.087</v>
       </c>
       <c r="E253" t="n">
         <v>49.5</v>
@@ -13846,19 +13846,19 @@
         <v>7.5</v>
       </c>
       <c r="H253" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I253" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="J253" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K253" t="n">
         <v>0</v>
       </c>
       <c r="L253" t="n">
-        <v>117.4867346938776</v>
+        <v>141.9255102040816</v>
       </c>
       <c r="M253" t="n">
         <v>55</v>
@@ -13887,7 +13887,7 @@
         <v>13</v>
       </c>
       <c r="D254" t="n">
-        <v>112.44</v>
+        <v>136.236</v>
       </c>
       <c r="E254" t="n">
         <v>56.911</v>
@@ -13899,19 +13899,19 @@
         <v>33.5</v>
       </c>
       <c r="H254" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I254" t="n">
-        <v>33.5</v>
+        <v>32</v>
       </c>
       <c r="J254" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K254" t="n">
         <v>0</v>
       </c>
       <c r="L254" t="n">
-        <v>114.734693877551</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M254" t="n">
         <v>63.23444444444445</v>
@@ -13940,7 +13940,7 @@
         <v>14</v>
       </c>
       <c r="D255" t="n">
-        <v>112.44</v>
+        <v>136.236</v>
       </c>
       <c r="E255" t="n">
         <v>56.911</v>
@@ -13952,19 +13952,19 @@
         <v>46</v>
       </c>
       <c r="H255" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I255" t="n">
-        <v>46</v>
+        <v>42.5</v>
       </c>
       <c r="J255" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K255" t="n">
         <v>0</v>
       </c>
       <c r="L255" t="n">
-        <v>114.734693877551</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M255" t="n">
         <v>63.23444444444445</v>
@@ -13993,7 +13993,7 @@
         <v>15</v>
       </c>
       <c r="D256" t="n">
-        <v>114.258</v>
+        <v>122.799</v>
       </c>
       <c r="E256" t="n">
         <v>53.581</v>
@@ -14005,10 +14005,10 @@
         <v>60</v>
       </c>
       <c r="H256" t="n">
-        <v>0.2846938775510068</v>
+        <v>9</v>
       </c>
       <c r="I256" t="n">
-        <v>59.71530612244899</v>
+        <v>51</v>
       </c>
       <c r="J256" t="n">
         <v>116.3051020408163</v>
@@ -14017,7 +14017,7 @@
         <v>0</v>
       </c>
       <c r="L256" t="n">
-        <v>116.5897959183673</v>
+        <v>125.3051020408163</v>
       </c>
       <c r="M256" t="n">
         <v>59.53444444444445</v>
@@ -14046,7 +14046,7 @@
         <v>16</v>
       </c>
       <c r="D257" t="n">
-        <v>131.363</v>
+        <v>140.444</v>
       </c>
       <c r="E257" t="n">
         <v>41.57</v>
@@ -14058,19 +14058,19 @@
         <v>77.5</v>
       </c>
       <c r="H257" t="n">
-        <v>13.5</v>
+        <v>11</v>
       </c>
       <c r="I257" t="n">
-        <v>64</v>
+        <v>66.5</v>
       </c>
       <c r="J257" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K257" t="n">
         <v>0</v>
       </c>
       <c r="L257" t="n">
-        <v>134.0438775510204</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M257" t="n">
         <v>46.18888888888889</v>
@@ -14099,7 +14099,7 @@
         <v>17</v>
       </c>
       <c r="D258" t="n">
-        <v>131.363</v>
+        <v>140.444</v>
       </c>
       <c r="E258" t="n">
         <v>41.57</v>
@@ -14111,19 +14111,19 @@
         <v>90</v>
       </c>
       <c r="H258" t="n">
-        <v>1.733673469387782</v>
+        <v>9</v>
       </c>
       <c r="I258" t="n">
-        <v>88.26632653061222</v>
+        <v>81</v>
       </c>
       <c r="J258" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K258" t="n">
         <v>0</v>
       </c>
       <c r="L258" t="n">
-        <v>134.0438775510204</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M258" t="n">
         <v>46.18888888888889</v>
@@ -14152,7 +14152,7 @@
         <v>18</v>
       </c>
       <c r="D259" t="n">
-        <v>94.574</v>
+        <v>122.803</v>
       </c>
       <c r="E259" t="n">
         <v>48.767</v>
@@ -14164,19 +14164,19 @@
         <v>86.5</v>
       </c>
       <c r="H259" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I259" t="n">
-        <v>86.5</v>
+        <v>81.5</v>
       </c>
       <c r="J259" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K259" t="n">
         <v>0</v>
       </c>
       <c r="L259" t="n">
-        <v>96.50408163265305</v>
+        <v>125.3091836734694</v>
       </c>
       <c r="M259" t="n">
         <v>54.18555555555556</v>
@@ -14205,7 +14205,7 @@
         <v>19</v>
       </c>
       <c r="D260" t="n">
-        <v>91.65600000000001</v>
+        <v>117.645</v>
       </c>
       <c r="E260" t="n">
         <v>43.091</v>
@@ -14217,19 +14217,19 @@
         <v>64.5</v>
       </c>
       <c r="H260" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="I260" t="n">
-        <v>64.5</v>
+        <v>61</v>
       </c>
       <c r="J260" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K260" t="n">
         <v>0</v>
       </c>
       <c r="L260" t="n">
-        <v>93.52653061224491</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M260" t="n">
         <v>47.87888888888889</v>
@@ -14258,7 +14258,7 @@
         <v>20</v>
       </c>
       <c r="D261" t="n">
-        <v>91.65600000000001</v>
+        <v>117.645</v>
       </c>
       <c r="E261" t="n">
         <v>43.091</v>
@@ -14279,10 +14279,10 @@
         <v>32.54591836734694</v>
       </c>
       <c r="K261" t="n">
-        <v>38.48061224489797</v>
+        <v>65</v>
       </c>
       <c r="L261" t="n">
-        <v>93.52653061224491</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M261" t="n">
         <v>47.87888888888889</v>
@@ -14311,7 +14311,7 @@
         <v>21</v>
       </c>
       <c r="D262" t="n">
-        <v>93.696</v>
+        <v>119.884</v>
       </c>
       <c r="E262" t="n">
         <v>44.625</v>
@@ -14332,10 +14332,10 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>87.60816326530612</v>
+        <v>114.330612244898</v>
       </c>
       <c r="L262" t="n">
-        <v>95.60816326530612</v>
+        <v>122.330612244898</v>
       </c>
       <c r="M262" t="n">
         <v>49.58333333333334</v>
@@ -14364,7 +14364,7 @@
         <v>22</v>
       </c>
       <c r="D263" t="n">
-        <v>98.786</v>
+        <v>110.043</v>
       </c>
       <c r="E263" t="n">
         <v>40.775</v>
@@ -14385,22 +14385,22 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>27.97142857142857</v>
+        <v>49.5</v>
       </c>
       <c r="L263" t="n">
-        <v>57.97142857142857</v>
+        <v>79.5</v>
       </c>
       <c r="M263" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N263" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O263" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P263" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q263" t="n">
         <v>0</v>
@@ -14417,7 +14417,7 @@
         <v>23</v>
       </c>
       <c r="D264" t="n">
-        <v>98.786</v>
+        <v>110.043</v>
       </c>
       <c r="E264" t="n">
         <v>40.775</v>
@@ -14438,10 +14438,10 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>13.51326530612243</v>
+        <v>25</v>
       </c>
       <c r="L264" t="n">
-        <v>60.01326530612243</v>
+        <v>71.5</v>
       </c>
       <c r="M264" t="n">
         <v>99.5898765432099</v>
@@ -14470,7 +14470,7 @@
         <v>24</v>
       </c>
       <c r="D265" t="n">
-        <v>97.666</v>
+        <v>102.145</v>
       </c>
       <c r="E265" t="n">
         <v>34.648</v>
@@ -14491,10 +14491,10 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>64.15918367346939</v>
+        <v>68.7295918367347</v>
       </c>
       <c r="L265" t="n">
-        <v>99.65918367346939</v>
+        <v>104.2295918367347</v>
       </c>
       <c r="M265" t="n">
         <v>38.49777777777778</v>
@@ -14523,7 +14523,7 @@
         <v>1</v>
       </c>
       <c r="D266" t="n">
-        <v>67.804</v>
+        <v>68.551</v>
       </c>
       <c r="E266" t="n">
         <v>35.363</v>
@@ -14544,10 +14544,10 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>57.18775510204082</v>
+        <v>57.95</v>
       </c>
       <c r="L266" t="n">
-        <v>69.18775510204082</v>
+        <v>69.95</v>
       </c>
       <c r="M266" t="n">
         <v>39.29222222222222</v>
@@ -14576,7 +14576,7 @@
         <v>2</v>
       </c>
       <c r="D267" t="n">
-        <v>67.804</v>
+        <v>68.551</v>
       </c>
       <c r="E267" t="n">
         <v>35.363</v>
@@ -14597,10 +14597,10 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>50.68775510204082</v>
+        <v>51.45</v>
       </c>
       <c r="L267" t="n">
-        <v>69.18775510204082</v>
+        <v>69.95</v>
       </c>
       <c r="M267" t="n">
         <v>39.29222222222222</v>
@@ -14629,7 +14629,7 @@
         <v>3</v>
       </c>
       <c r="D268" t="n">
-        <v>67.804</v>
+        <v>68.551</v>
       </c>
       <c r="E268" t="n">
         <v>35.363</v>
@@ -14650,10 +14650,10 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>46.68775510204082</v>
+        <v>47.45</v>
       </c>
       <c r="L268" t="n">
-        <v>69.18775510204082</v>
+        <v>69.95</v>
       </c>
       <c r="M268" t="n">
         <v>39.29222222222222</v>
@@ -14682,7 +14682,7 @@
         <v>4</v>
       </c>
       <c r="D269" t="n">
-        <v>67.804</v>
+        <v>68.483</v>
       </c>
       <c r="E269" t="n">
         <v>38.078</v>
@@ -14703,10 +14703,10 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>42.18775510204082</v>
+        <v>42.88061224489796</v>
       </c>
       <c r="L269" t="n">
-        <v>69.18775510204082</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M269" t="n">
         <v>42.30888888888889</v>
@@ -14735,7 +14735,7 @@
         <v>5</v>
       </c>
       <c r="D270" t="n">
-        <v>67.804</v>
+        <v>68.483</v>
       </c>
       <c r="E270" t="n">
         <v>38.078</v>
@@ -14756,10 +14756,10 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>38.68775510204082</v>
+        <v>39.38061224489796</v>
       </c>
       <c r="L270" t="n">
-        <v>69.18775510204082</v>
+        <v>69.88061224489796</v>
       </c>
       <c r="M270" t="n">
         <v>42.30888888888889</v>
@@ -14788,7 +14788,7 @@
         <v>6</v>
       </c>
       <c r="D271" t="n">
-        <v>75.039</v>
+        <v>75.066</v>
       </c>
       <c r="E271" t="n">
         <v>38.078</v>
@@ -14809,10 +14809,10 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>56.07040816326531</v>
+        <v>56.09795918367347</v>
       </c>
       <c r="L271" t="n">
-        <v>76.57040816326531</v>
+        <v>76.59795918367347</v>
       </c>
       <c r="M271" t="n">
         <v>42.30888888888889</v>
@@ -14841,7 +14841,7 @@
         <v>7</v>
       </c>
       <c r="D272" t="n">
-        <v>78.58799999999999</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E272" t="n">
         <v>48.821</v>
@@ -14862,10 +14862,10 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>62.69183673469388</v>
+        <v>68.33469387755102</v>
       </c>
       <c r="L272" t="n">
-        <v>80.19183673469388</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M272" t="n">
         <v>54.24555555555555</v>
@@ -14894,7 +14894,7 @@
         <v>8</v>
       </c>
       <c r="D273" t="n">
-        <v>78.58799999999999</v>
+        <v>84.11799999999999</v>
       </c>
       <c r="E273" t="n">
         <v>48.821</v>
@@ -14915,10 +14915,10 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>65.19183673469388</v>
+        <v>70.83469387755102</v>
       </c>
       <c r="L273" t="n">
-        <v>80.19183673469388</v>
+        <v>85.83469387755102</v>
       </c>
       <c r="M273" t="n">
         <v>54.24555555555555</v>
@@ -14947,7 +14947,7 @@
         <v>9</v>
       </c>
       <c r="D274" t="n">
-        <v>118.618</v>
+        <v>125.853</v>
       </c>
       <c r="E274" t="n">
         <v>61.411</v>
@@ -14968,10 +14968,10 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>111.0387755102041</v>
+        <v>118.4214285714286</v>
       </c>
       <c r="L274" t="n">
-        <v>121.0387755102041</v>
+        <v>128.4214285714286</v>
       </c>
       <c r="M274" t="n">
         <v>68.23444444444445</v>
@@ -15000,7 +15000,7 @@
         <v>10</v>
       </c>
       <c r="D275" t="n">
-        <v>116.928</v>
+        <v>138.408</v>
       </c>
       <c r="E275" t="n">
         <v>45.383</v>
@@ -15018,13 +15018,13 @@
         <v>0</v>
       </c>
       <c r="J275" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="K275" t="n">
-        <v>38.39285714285714</v>
+        <v>47.5</v>
       </c>
       <c r="L275" t="n">
-        <v>119.3142857142857</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M275" t="n">
         <v>50.42555555555556</v>
@@ -15053,7 +15053,7 @@
         <v>11</v>
       </c>
       <c r="D276" t="n">
-        <v>116.928</v>
+        <v>138.408</v>
       </c>
       <c r="E276" t="n">
         <v>45.383</v>
@@ -15065,19 +15065,19 @@
         <v>1</v>
       </c>
       <c r="H276" t="n">
-        <v>-0</v>
+        <v>0.5</v>
       </c>
       <c r="I276" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J276" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="K276" t="n">
         <v>0</v>
       </c>
       <c r="L276" t="n">
-        <v>119.3142857142857</v>
+        <v>141.2326530612245</v>
       </c>
       <c r="M276" t="n">
         <v>50.42555555555556</v>
@@ -15106,7 +15106,7 @@
         <v>12</v>
       </c>
       <c r="D277" t="n">
-        <v>115.137</v>
+        <v>139.087</v>
       </c>
       <c r="E277" t="n">
         <v>49.5</v>
@@ -15118,19 +15118,19 @@
         <v>1</v>
       </c>
       <c r="H277" t="n">
-        <v>-0</v>
+        <v>1</v>
       </c>
       <c r="I277" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J277" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="K277" t="n">
         <v>0</v>
       </c>
       <c r="L277" t="n">
-        <v>117.4867346938776</v>
+        <v>141.9255102040816</v>
       </c>
       <c r="M277" t="n">
         <v>55</v>
@@ -15145,7 +15145,7 @@
         <v>49.5</v>
       </c>
       <c r="Q277" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="278">
@@ -15159,7 +15159,7 @@
         <v>13</v>
       </c>
       <c r="D278" t="n">
-        <v>112.44</v>
+        <v>136.236</v>
       </c>
       <c r="E278" t="n">
         <v>56.911</v>
@@ -15171,19 +15171,19 @@
         <v>1.5</v>
       </c>
       <c r="H278" t="n">
-        <v>-0</v>
+        <v>1.5</v>
       </c>
       <c r="I278" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="J278" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="K278" t="n">
         <v>0</v>
       </c>
       <c r="L278" t="n">
-        <v>114.734693877551</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M278" t="n">
         <v>63.23444444444445</v>
@@ -15198,7 +15198,7 @@
         <v>56.91100000000001</v>
       </c>
       <c r="Q278" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="279">
@@ -15212,7 +15212,7 @@
         <v>14</v>
       </c>
       <c r="D279" t="n">
-        <v>112.44</v>
+        <v>136.236</v>
       </c>
       <c r="E279" t="n">
         <v>56.911</v>
@@ -15224,19 +15224,19 @@
         <v>6</v>
       </c>
       <c r="H279" t="n">
-        <v>-0</v>
+        <v>3.5</v>
       </c>
       <c r="I279" t="n">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="J279" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="K279" t="n">
         <v>0</v>
       </c>
       <c r="L279" t="n">
-        <v>114.734693877551</v>
+        <v>139.0163265306122</v>
       </c>
       <c r="M279" t="n">
         <v>63.23444444444445</v>
@@ -15265,7 +15265,7 @@
         <v>15</v>
       </c>
       <c r="D280" t="n">
-        <v>114.258</v>
+        <v>122.799</v>
       </c>
       <c r="E280" t="n">
         <v>53.581</v>
@@ -15277,10 +15277,10 @@
         <v>13</v>
       </c>
       <c r="H280" t="n">
-        <v>0.2846938775510068</v>
+        <v>9</v>
       </c>
       <c r="I280" t="n">
-        <v>12.71530612244899</v>
+        <v>4</v>
       </c>
       <c r="J280" t="n">
         <v>116.3051020408163</v>
@@ -15289,7 +15289,7 @@
         <v>0</v>
       </c>
       <c r="L280" t="n">
-        <v>116.5897959183673</v>
+        <v>125.3051020408163</v>
       </c>
       <c r="M280" t="n">
         <v>59.53444444444445</v>
@@ -15318,7 +15318,7 @@
         <v>16</v>
       </c>
       <c r="D281" t="n">
-        <v>131.363</v>
+        <v>140.444</v>
       </c>
       <c r="E281" t="n">
         <v>41.57</v>
@@ -15330,19 +15330,19 @@
         <v>13.5</v>
       </c>
       <c r="H281" t="n">
-        <v>13.5</v>
+        <v>11</v>
       </c>
       <c r="I281" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="J281" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="K281" t="n">
         <v>0</v>
       </c>
       <c r="L281" t="n">
-        <v>134.0438775510204</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M281" t="n">
         <v>46.18888888888889</v>
@@ -15357,7 +15357,7 @@
         <v>41.57</v>
       </c>
       <c r="Q281" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="282">
@@ -15371,7 +15371,7 @@
         <v>17</v>
       </c>
       <c r="D282" t="n">
-        <v>131.363</v>
+        <v>140.444</v>
       </c>
       <c r="E282" t="n">
         <v>41.57</v>
@@ -15383,19 +15383,19 @@
         <v>9</v>
       </c>
       <c r="H282" t="n">
-        <v>1.733673469387782</v>
+        <v>9</v>
       </c>
       <c r="I282" t="n">
-        <v>7.266326530612218</v>
+        <v>0</v>
       </c>
       <c r="J282" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="K282" t="n">
         <v>0</v>
       </c>
       <c r="L282" t="n">
-        <v>134.0438775510204</v>
+        <v>143.3102040816326</v>
       </c>
       <c r="M282" t="n">
         <v>46.18888888888889</v>
@@ -15410,7 +15410,7 @@
         <v>41.57</v>
       </c>
       <c r="Q282" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283">
@@ -15424,7 +15424,7 @@
         <v>18</v>
       </c>
       <c r="D283" t="n">
-        <v>94.574</v>
+        <v>122.803</v>
       </c>
       <c r="E283" t="n">
         <v>48.767</v>
@@ -15436,19 +15436,19 @@
         <v>5</v>
       </c>
       <c r="H283" t="n">
-        <v>-0</v>
+        <v>5</v>
       </c>
       <c r="I283" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J283" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="K283" t="n">
         <v>0</v>
       </c>
       <c r="L283" t="n">
-        <v>96.50408163265305</v>
+        <v>125.3091836734694</v>
       </c>
       <c r="M283" t="n">
         <v>54.18555555555556</v>
@@ -15463,7 +15463,7 @@
         <v>48.767</v>
       </c>
       <c r="Q283" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="284">
@@ -15477,7 +15477,7 @@
         <v>19</v>
       </c>
       <c r="D284" t="n">
-        <v>91.65600000000001</v>
+        <v>117.645</v>
       </c>
       <c r="E284" t="n">
         <v>43.091</v>
@@ -15489,19 +15489,19 @@
         <v>3.5</v>
       </c>
       <c r="H284" t="n">
-        <v>-0</v>
+        <v>3.5</v>
       </c>
       <c r="I284" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="J284" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="K284" t="n">
         <v>0</v>
       </c>
       <c r="L284" t="n">
-        <v>93.52653061224491</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M284" t="n">
         <v>47.87888888888889</v>
@@ -15516,7 +15516,7 @@
         <v>43.09100000000001</v>
       </c>
       <c r="Q284" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="285">
@@ -15530,7 +15530,7 @@
         <v>20</v>
       </c>
       <c r="D285" t="n">
-        <v>91.65600000000001</v>
+        <v>117.645</v>
       </c>
       <c r="E285" t="n">
         <v>43.091</v>
@@ -15551,10 +15551,10 @@
         <v>32.54591836734694</v>
       </c>
       <c r="K285" t="n">
-        <v>56.98061224489797</v>
+        <v>83.5</v>
       </c>
       <c r="L285" t="n">
-        <v>93.52653061224491</v>
+        <v>120.0459183673469</v>
       </c>
       <c r="M285" t="n">
         <v>47.87888888888889</v>
@@ -15583,7 +15583,7 @@
         <v>21</v>
       </c>
       <c r="D286" t="n">
-        <v>93.696</v>
+        <v>119.884</v>
       </c>
       <c r="E286" t="n">
         <v>44.625</v>
@@ -15604,10 +15604,10 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>92.60816326530612</v>
+        <v>119.330612244898</v>
       </c>
       <c r="L286" t="n">
-        <v>95.60816326530612</v>
+        <v>122.330612244898</v>
       </c>
       <c r="M286" t="n">
         <v>49.58333333333334</v>
@@ -15636,7 +15636,7 @@
         <v>22</v>
       </c>
       <c r="D287" t="n">
-        <v>98.786</v>
+        <v>110.043</v>
       </c>
       <c r="E287" t="n">
         <v>40.775</v>
@@ -15657,22 +15657,22 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>53.97142857142857</v>
+        <v>75.5</v>
       </c>
       <c r="L287" t="n">
-        <v>57.97142857142857</v>
+        <v>79.5</v>
       </c>
       <c r="M287" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="N287" t="n">
-        <v>93.27555555555556</v>
+        <v>71.40666666666671</v>
       </c>
       <c r="O287" t="n">
-        <v>9.031728395061734</v>
+        <v>17.53629629629627</v>
       </c>
       <c r="P287" t="n">
-        <v>8.128555555555561</v>
+        <v>15.78266666666664</v>
       </c>
       <c r="Q287" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>23</v>
       </c>
       <c r="D288" t="n">
-        <v>98.786</v>
+        <v>110.043</v>
       </c>
       <c r="E288" t="n">
         <v>40.775</v>
@@ -15710,10 +15710,10 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>50.01326530612243</v>
+        <v>61.5</v>
       </c>
       <c r="L288" t="n">
-        <v>60.01326530612243</v>
+        <v>71.5</v>
       </c>
       <c r="M288" t="n">
         <v>99.5898765432099</v>
@@ -15742,7 +15742,7 @@
         <v>24</v>
       </c>
       <c r="D289" t="n">
-        <v>97.666</v>
+        <v>102.145</v>
       </c>
       <c r="E289" t="n">
         <v>34.648</v>
@@ -15763,10 +15763,10 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>84.65918367346939</v>
+        <v>89.2295918367347</v>
       </c>
       <c r="L289" t="n">
-        <v>99.65918367346939</v>
+        <v>104.2295918367347</v>
       </c>
       <c r="M289" t="n">
         <v>38.49777777777778</v>
@@ -15983,7 +15983,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>77.92142857142858</v>
+        <v>90.73265306122448</v>
       </c>
       <c r="C11" t="n">
         <v>50.42555555555556</v>
@@ -16000,7 +16000,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>119.3142857142857</v>
+        <v>140.7326530612245</v>
       </c>
       <c r="C12" t="n">
         <v>50.42555555555556</v>
@@ -16017,7 +16017,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>117.4867346938776</v>
+        <v>140.9255102040816</v>
       </c>
       <c r="C13" t="n">
         <v>55</v>
@@ -16034,7 +16034,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>114.734693877551</v>
+        <v>137.5163265306122</v>
       </c>
       <c r="C14" t="n">
         <v>63.23444444444445</v>
@@ -16051,7 +16051,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>114.734693877551</v>
+        <v>135.5163265306122</v>
       </c>
       <c r="C15" t="n">
         <v>63.23444444444445</v>
@@ -16085,7 +16085,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>120.5438775510204</v>
+        <v>132.3102040816326</v>
       </c>
       <c r="C17" t="n">
         <v>46.18888888888889</v>
@@ -16102,7 +16102,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>132.3102040816326</v>
+        <v>134.3102040816326</v>
       </c>
       <c r="C18" t="n">
         <v>46.18888888888889</v>
@@ -16119,7 +16119,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>96.50408163265305</v>
+        <v>120.3091836734694</v>
       </c>
       <c r="C19" t="n">
         <v>54.18555555555556</v>
@@ -16136,7 +16136,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>93.52653061224491</v>
+        <v>116.5459183673469</v>
       </c>
       <c r="C20" t="n">
         <v>47.87888888888889</v>
@@ -16190,7 +16190,7 @@
         <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>102.3072839506173</v>
+        <v>88.94296296296298</v>
       </c>
       <c r="D23" t="n">
         <v>129.17</v>

</xml_diff>